<commit_message>
Add FASASI entries; normalize PRACTICAL values
Added two FASASI codes (FAS1122, FAS1123) to code_registry.json and corresponding student records to students_1st_term.json with fees and payments. Normalized PRACTICAL fields across students (e.g., "0.0" -> "0", "3750.0" -> "3750") and updated payment totals/balances for affected students (notably FAGBAYI ASEOLUWA JOSHUA and JAMIU FAIZAH AYANFE). Updated binary Excel files (2026 - 2027 FEE.xlsx, parent_codes.xlsx) as well.
</commit_message>
<xml_diff>
--- a/parent_codes.xlsx
+++ b/parent_codes.xlsx
@@ -14,7 +14,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="360" uniqueCount="256">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="366" uniqueCount="259">
   <si>
     <t>Code</t>
   </si>
@@ -184,6 +184,12 @@
     <t>FAGASE1053</t>
   </si>
   <si>
+    <t>FAS1122</t>
+  </si>
+  <si>
+    <t>FAS1123</t>
+  </si>
+  <si>
     <t>FEYJAD1054</t>
   </si>
   <si>
@@ -539,6 +545,9 @@
   </si>
   <si>
     <t>FAGBAYI ASEOLUWA JOSHUA</t>
+  </si>
+  <si>
+    <t>FASASI</t>
   </si>
   <si>
     <t>FEYIJIMI JADEN OLAOLUWA</t>
@@ -1113,7 +1122,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C120"/>
+  <dimension ref="A1:C122"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:3">
@@ -1132,10 +1141,10 @@
         <v>3</v>
       </c>
       <c r="B2" t="s">
-        <v>122</v>
+        <v>124</v>
       </c>
       <c r="C2" t="s">
-        <v>241</v>
+        <v>244</v>
       </c>
     </row>
     <row r="3" spans="1:3">
@@ -1143,10 +1152,10 @@
         <v>4</v>
       </c>
       <c r="B3" t="s">
-        <v>123</v>
+        <v>125</v>
       </c>
       <c r="C3" t="s">
-        <v>242</v>
+        <v>245</v>
       </c>
     </row>
     <row r="4" spans="1:3">
@@ -1154,10 +1163,10 @@
         <v>5</v>
       </c>
       <c r="B4" t="s">
-        <v>124</v>
+        <v>126</v>
       </c>
       <c r="C4" t="s">
-        <v>243</v>
+        <v>246</v>
       </c>
     </row>
     <row r="5" spans="1:3">
@@ -1165,10 +1174,10 @@
         <v>6</v>
       </c>
       <c r="B5" t="s">
-        <v>125</v>
+        <v>127</v>
       </c>
       <c r="C5" t="s">
-        <v>244</v>
+        <v>247</v>
       </c>
     </row>
     <row r="6" spans="1:3">
@@ -1176,10 +1185,10 @@
         <v>7</v>
       </c>
       <c r="B6" t="s">
-        <v>126</v>
+        <v>128</v>
       </c>
       <c r="C6" t="s">
-        <v>241</v>
+        <v>244</v>
       </c>
     </row>
     <row r="7" spans="1:3">
@@ -1187,10 +1196,10 @@
         <v>8</v>
       </c>
       <c r="B7" t="s">
-        <v>127</v>
+        <v>129</v>
       </c>
       <c r="C7" t="s">
-        <v>245</v>
+        <v>248</v>
       </c>
     </row>
     <row r="8" spans="1:3">
@@ -1198,10 +1207,10 @@
         <v>9</v>
       </c>
       <c r="B8" t="s">
-        <v>128</v>
+        <v>130</v>
       </c>
       <c r="C8" t="s">
-        <v>246</v>
+        <v>249</v>
       </c>
     </row>
     <row r="9" spans="1:3">
@@ -1209,10 +1218,10 @@
         <v>10</v>
       </c>
       <c r="B9" t="s">
-        <v>129</v>
+        <v>131</v>
       </c>
       <c r="C9" t="s">
-        <v>245</v>
+        <v>248</v>
       </c>
     </row>
     <row r="10" spans="1:3">
@@ -1220,10 +1229,10 @@
         <v>11</v>
       </c>
       <c r="B10" t="s">
-        <v>130</v>
+        <v>132</v>
       </c>
       <c r="C10" t="s">
-        <v>245</v>
+        <v>248</v>
       </c>
     </row>
     <row r="11" spans="1:3">
@@ -1231,10 +1240,10 @@
         <v>12</v>
       </c>
       <c r="B11" t="s">
-        <v>131</v>
+        <v>133</v>
       </c>
       <c r="C11" t="s">
-        <v>245</v>
+        <v>248</v>
       </c>
     </row>
     <row r="12" spans="1:3">
@@ -1242,10 +1251,10 @@
         <v>13</v>
       </c>
       <c r="B12" t="s">
-        <v>132</v>
+        <v>134</v>
       </c>
       <c r="C12" t="s">
-        <v>244</v>
+        <v>247</v>
       </c>
     </row>
     <row r="13" spans="1:3">
@@ -1253,10 +1262,10 @@
         <v>14</v>
       </c>
       <c r="B13" t="s">
-        <v>133</v>
+        <v>135</v>
       </c>
       <c r="C13" t="s">
-        <v>246</v>
+        <v>249</v>
       </c>
     </row>
     <row r="14" spans="1:3">
@@ -1264,10 +1273,10 @@
         <v>15</v>
       </c>
       <c r="B14" t="s">
-        <v>134</v>
+        <v>136</v>
       </c>
       <c r="C14" t="s">
-        <v>243</v>
+        <v>246</v>
       </c>
     </row>
     <row r="15" spans="1:3">
@@ -1275,10 +1284,10 @@
         <v>16</v>
       </c>
       <c r="B15" t="s">
-        <v>135</v>
+        <v>137</v>
       </c>
       <c r="C15" t="s">
-        <v>242</v>
+        <v>245</v>
       </c>
     </row>
     <row r="16" spans="1:3">
@@ -1286,10 +1295,10 @@
         <v>17</v>
       </c>
       <c r="B16" t="s">
-        <v>136</v>
+        <v>138</v>
       </c>
       <c r="C16" t="s">
-        <v>246</v>
+        <v>249</v>
       </c>
     </row>
     <row r="17" spans="1:3">
@@ -1297,10 +1306,10 @@
         <v>18</v>
       </c>
       <c r="B17" t="s">
-        <v>137</v>
+        <v>139</v>
       </c>
       <c r="C17" t="s">
-        <v>244</v>
+        <v>247</v>
       </c>
     </row>
     <row r="18" spans="1:3">
@@ -1308,10 +1317,10 @@
         <v>19</v>
       </c>
       <c r="B18" t="s">
-        <v>138</v>
+        <v>140</v>
       </c>
       <c r="C18" t="s">
-        <v>247</v>
+        <v>250</v>
       </c>
     </row>
     <row r="19" spans="1:3">
@@ -1319,10 +1328,10 @@
         <v>20</v>
       </c>
       <c r="B19" t="s">
-        <v>139</v>
+        <v>141</v>
       </c>
       <c r="C19" t="s">
-        <v>242</v>
+        <v>245</v>
       </c>
     </row>
     <row r="20" spans="1:3">
@@ -1330,10 +1339,10 @@
         <v>21</v>
       </c>
       <c r="B20" t="s">
-        <v>140</v>
+        <v>142</v>
       </c>
       <c r="C20" t="s">
-        <v>248</v>
+        <v>251</v>
       </c>
     </row>
     <row r="21" spans="1:3">
@@ -1341,10 +1350,10 @@
         <v>22</v>
       </c>
       <c r="B21" t="s">
-        <v>141</v>
+        <v>143</v>
       </c>
       <c r="C21" t="s">
-        <v>245</v>
+        <v>248</v>
       </c>
     </row>
     <row r="22" spans="1:3">
@@ -1352,10 +1361,10 @@
         <v>23</v>
       </c>
       <c r="B22" t="s">
-        <v>142</v>
+        <v>144</v>
       </c>
       <c r="C22" t="s">
-        <v>249</v>
+        <v>252</v>
       </c>
     </row>
     <row r="23" spans="1:3">
@@ -1363,10 +1372,10 @@
         <v>24</v>
       </c>
       <c r="B23" t="s">
-        <v>143</v>
+        <v>145</v>
       </c>
       <c r="C23" t="s">
-        <v>250</v>
+        <v>253</v>
       </c>
     </row>
     <row r="24" spans="1:3">
@@ -1374,10 +1383,10 @@
         <v>25</v>
       </c>
       <c r="B24" t="s">
-        <v>144</v>
+        <v>146</v>
       </c>
       <c r="C24" t="s">
-        <v>249</v>
+        <v>252</v>
       </c>
     </row>
     <row r="25" spans="1:3">
@@ -1385,10 +1394,10 @@
         <v>26</v>
       </c>
       <c r="B25" t="s">
-        <v>145</v>
+        <v>147</v>
       </c>
       <c r="C25" t="s">
-        <v>245</v>
+        <v>248</v>
       </c>
     </row>
     <row r="26" spans="1:3">
@@ -1396,10 +1405,10 @@
         <v>27</v>
       </c>
       <c r="B26" t="s">
-        <v>146</v>
+        <v>148</v>
       </c>
       <c r="C26" t="s">
-        <v>251</v>
+        <v>254</v>
       </c>
     </row>
     <row r="27" spans="1:3">
@@ -1407,10 +1416,10 @@
         <v>28</v>
       </c>
       <c r="B27" t="s">
-        <v>147</v>
+        <v>149</v>
       </c>
       <c r="C27" t="s">
-        <v>250</v>
+        <v>253</v>
       </c>
     </row>
     <row r="28" spans="1:3">
@@ -1418,10 +1427,10 @@
         <v>29</v>
       </c>
       <c r="B28" t="s">
-        <v>148</v>
+        <v>150</v>
       </c>
       <c r="C28" t="s">
-        <v>252</v>
+        <v>255</v>
       </c>
     </row>
     <row r="29" spans="1:3">
@@ -1429,10 +1438,10 @@
         <v>30</v>
       </c>
       <c r="B29" t="s">
-        <v>149</v>
+        <v>151</v>
       </c>
       <c r="C29" t="s">
-        <v>247</v>
+        <v>250</v>
       </c>
     </row>
     <row r="30" spans="1:3">
@@ -1440,10 +1449,10 @@
         <v>31</v>
       </c>
       <c r="B30" t="s">
-        <v>150</v>
+        <v>152</v>
       </c>
       <c r="C30" t="s">
-        <v>247</v>
+        <v>250</v>
       </c>
     </row>
     <row r="31" spans="1:3">
@@ -1451,10 +1460,10 @@
         <v>32</v>
       </c>
       <c r="B31" t="s">
-        <v>151</v>
+        <v>153</v>
       </c>
       <c r="C31" t="s">
-        <v>249</v>
+        <v>252</v>
       </c>
     </row>
     <row r="32" spans="1:3">
@@ -1462,10 +1471,10 @@
         <v>33</v>
       </c>
       <c r="B32" t="s">
-        <v>152</v>
+        <v>154</v>
       </c>
       <c r="C32" t="s">
-        <v>253</v>
+        <v>256</v>
       </c>
     </row>
     <row r="33" spans="1:3">
@@ -1473,10 +1482,10 @@
         <v>34</v>
       </c>
       <c r="B33" t="s">
-        <v>153</v>
+        <v>155</v>
       </c>
       <c r="C33" t="s">
-        <v>241</v>
+        <v>244</v>
       </c>
     </row>
     <row r="34" spans="1:3">
@@ -1484,10 +1493,10 @@
         <v>35</v>
       </c>
       <c r="B34" t="s">
-        <v>154</v>
+        <v>156</v>
       </c>
       <c r="C34" t="s">
-        <v>242</v>
+        <v>245</v>
       </c>
     </row>
     <row r="35" spans="1:3">
@@ -1495,10 +1504,10 @@
         <v>36</v>
       </c>
       <c r="B35" t="s">
-        <v>155</v>
+        <v>157</v>
       </c>
       <c r="C35" t="s">
-        <v>241</v>
+        <v>244</v>
       </c>
     </row>
     <row r="36" spans="1:3">
@@ -1506,10 +1515,10 @@
         <v>37</v>
       </c>
       <c r="B36" t="s">
-        <v>156</v>
+        <v>158</v>
       </c>
       <c r="C36" t="s">
-        <v>244</v>
+        <v>247</v>
       </c>
     </row>
     <row r="37" spans="1:3">
@@ -1517,10 +1526,10 @@
         <v>38</v>
       </c>
       <c r="B37" t="s">
-        <v>157</v>
+        <v>159</v>
       </c>
       <c r="C37" t="s">
-        <v>249</v>
+        <v>252</v>
       </c>
     </row>
     <row r="38" spans="1:3">
@@ -1528,10 +1537,10 @@
         <v>39</v>
       </c>
       <c r="B38" t="s">
-        <v>158</v>
+        <v>160</v>
       </c>
       <c r="C38" t="s">
-        <v>253</v>
+        <v>256</v>
       </c>
     </row>
     <row r="39" spans="1:3">
@@ -1539,10 +1548,10 @@
         <v>40</v>
       </c>
       <c r="B39" t="s">
-        <v>159</v>
+        <v>161</v>
       </c>
       <c r="C39" t="s">
-        <v>249</v>
+        <v>252</v>
       </c>
     </row>
     <row r="40" spans="1:3">
@@ -1550,10 +1559,10 @@
         <v>41</v>
       </c>
       <c r="B40" t="s">
-        <v>160</v>
+        <v>162</v>
       </c>
       <c r="C40" t="s">
-        <v>250</v>
+        <v>253</v>
       </c>
     </row>
     <row r="41" spans="1:3">
@@ -1561,10 +1570,10 @@
         <v>42</v>
       </c>
       <c r="B41" t="s">
-        <v>161</v>
+        <v>163</v>
       </c>
       <c r="C41" t="s">
-        <v>250</v>
+        <v>253</v>
       </c>
     </row>
     <row r="42" spans="1:3">
@@ -1572,10 +1581,10 @@
         <v>43</v>
       </c>
       <c r="B42" t="s">
-        <v>162</v>
+        <v>164</v>
       </c>
       <c r="C42" t="s">
-        <v>243</v>
+        <v>246</v>
       </c>
     </row>
     <row r="43" spans="1:3">
@@ -1583,10 +1592,10 @@
         <v>44</v>
       </c>
       <c r="B43" t="s">
-        <v>163</v>
+        <v>165</v>
       </c>
       <c r="C43" t="s">
-        <v>250</v>
+        <v>253</v>
       </c>
     </row>
     <row r="44" spans="1:3">
@@ -1594,10 +1603,10 @@
         <v>45</v>
       </c>
       <c r="B44" t="s">
-        <v>164</v>
+        <v>166</v>
       </c>
       <c r="C44" t="s">
-        <v>250</v>
+        <v>253</v>
       </c>
     </row>
     <row r="45" spans="1:3">
@@ -1605,10 +1614,10 @@
         <v>46</v>
       </c>
       <c r="B45" t="s">
-        <v>165</v>
+        <v>167</v>
       </c>
       <c r="C45" t="s">
-        <v>243</v>
+        <v>246</v>
       </c>
     </row>
     <row r="46" spans="1:3">
@@ -1616,10 +1625,10 @@
         <v>47</v>
       </c>
       <c r="B46" t="s">
-        <v>166</v>
+        <v>168</v>
       </c>
       <c r="C46" t="s">
-        <v>249</v>
+        <v>252</v>
       </c>
     </row>
     <row r="47" spans="1:3">
@@ -1627,10 +1636,10 @@
         <v>48</v>
       </c>
       <c r="B47" t="s">
-        <v>167</v>
+        <v>169</v>
       </c>
       <c r="C47" t="s">
-        <v>252</v>
+        <v>255</v>
       </c>
     </row>
     <row r="48" spans="1:3">
@@ -1638,10 +1647,10 @@
         <v>49</v>
       </c>
       <c r="B48" t="s">
-        <v>168</v>
+        <v>170</v>
       </c>
       <c r="C48" t="s">
-        <v>244</v>
+        <v>247</v>
       </c>
     </row>
     <row r="49" spans="1:3">
@@ -1649,10 +1658,10 @@
         <v>50</v>
       </c>
       <c r="B49" t="s">
-        <v>169</v>
+        <v>171</v>
       </c>
       <c r="C49" t="s">
-        <v>251</v>
+        <v>254</v>
       </c>
     </row>
     <row r="50" spans="1:3">
@@ -1660,10 +1669,10 @@
         <v>51</v>
       </c>
       <c r="B50" t="s">
-        <v>170</v>
+        <v>172</v>
       </c>
       <c r="C50" t="s">
-        <v>250</v>
+        <v>253</v>
       </c>
     </row>
     <row r="51" spans="1:3">
@@ -1671,10 +1680,10 @@
         <v>52</v>
       </c>
       <c r="B51" t="s">
-        <v>171</v>
+        <v>173</v>
       </c>
       <c r="C51" t="s">
-        <v>252</v>
+        <v>255</v>
       </c>
     </row>
     <row r="52" spans="1:3">
@@ -1682,10 +1691,10 @@
         <v>53</v>
       </c>
       <c r="B52" t="s">
-        <v>172</v>
+        <v>174</v>
       </c>
       <c r="C52" t="s">
-        <v>242</v>
+        <v>245</v>
       </c>
     </row>
     <row r="53" spans="1:3">
@@ -1693,10 +1702,10 @@
         <v>54</v>
       </c>
       <c r="B53" t="s">
-        <v>173</v>
+        <v>175</v>
       </c>
       <c r="C53" t="s">
-        <v>245</v>
+        <v>248</v>
       </c>
     </row>
     <row r="54" spans="1:3">
@@ -1704,10 +1713,10 @@
         <v>55</v>
       </c>
       <c r="B54" t="s">
-        <v>174</v>
+        <v>176</v>
       </c>
       <c r="C54" t="s">
-        <v>249</v>
+        <v>252</v>
       </c>
     </row>
     <row r="55" spans="1:3">
@@ -1715,10 +1724,10 @@
         <v>56</v>
       </c>
       <c r="B55" t="s">
-        <v>175</v>
+        <v>177</v>
       </c>
       <c r="C55" t="s">
-        <v>241</v>
+        <v>253</v>
       </c>
     </row>
     <row r="56" spans="1:3">
@@ -1726,7 +1735,7 @@
         <v>57</v>
       </c>
       <c r="B56" t="s">
-        <v>176</v>
+        <v>177</v>
       </c>
       <c r="C56" t="s">
         <v>251</v>
@@ -1737,10 +1746,10 @@
         <v>58</v>
       </c>
       <c r="B57" t="s">
-        <v>177</v>
+        <v>178</v>
       </c>
       <c r="C57" t="s">
-        <v>241</v>
+        <v>244</v>
       </c>
     </row>
     <row r="58" spans="1:3">
@@ -1748,10 +1757,10 @@
         <v>59</v>
       </c>
       <c r="B58" t="s">
-        <v>178</v>
+        <v>179</v>
       </c>
       <c r="C58" t="s">
-        <v>241</v>
+        <v>254</v>
       </c>
     </row>
     <row r="59" spans="1:3">
@@ -1759,10 +1768,10 @@
         <v>60</v>
       </c>
       <c r="B59" t="s">
-        <v>179</v>
+        <v>180</v>
       </c>
       <c r="C59" t="s">
-        <v>251</v>
+        <v>244</v>
       </c>
     </row>
     <row r="60" spans="1:3">
@@ -1770,10 +1779,10 @@
         <v>61</v>
       </c>
       <c r="B60" t="s">
-        <v>180</v>
+        <v>181</v>
       </c>
       <c r="C60" t="s">
-        <v>246</v>
+        <v>244</v>
       </c>
     </row>
     <row r="61" spans="1:3">
@@ -1781,10 +1790,10 @@
         <v>62</v>
       </c>
       <c r="B61" t="s">
-        <v>181</v>
+        <v>182</v>
       </c>
       <c r="C61" t="s">
-        <v>250</v>
+        <v>254</v>
       </c>
     </row>
     <row r="62" spans="1:3">
@@ -1792,10 +1801,10 @@
         <v>63</v>
       </c>
       <c r="B62" t="s">
-        <v>182</v>
+        <v>183</v>
       </c>
       <c r="C62" t="s">
-        <v>254</v>
+        <v>249</v>
       </c>
     </row>
     <row r="63" spans="1:3">
@@ -1803,10 +1812,10 @@
         <v>64</v>
       </c>
       <c r="B63" t="s">
-        <v>183</v>
+        <v>184</v>
       </c>
       <c r="C63" t="s">
-        <v>247</v>
+        <v>253</v>
       </c>
     </row>
     <row r="64" spans="1:3">
@@ -1814,10 +1823,10 @@
         <v>65</v>
       </c>
       <c r="B64" t="s">
-        <v>184</v>
+        <v>185</v>
       </c>
       <c r="C64" t="s">
-        <v>249</v>
+        <v>257</v>
       </c>
     </row>
     <row r="65" spans="1:3">
@@ -1825,10 +1834,10 @@
         <v>66</v>
       </c>
       <c r="B65" t="s">
-        <v>185</v>
+        <v>186</v>
       </c>
       <c r="C65" t="s">
-        <v>254</v>
+        <v>250</v>
       </c>
     </row>
     <row r="66" spans="1:3">
@@ -1836,10 +1845,10 @@
         <v>67</v>
       </c>
       <c r="B66" t="s">
-        <v>186</v>
+        <v>187</v>
       </c>
       <c r="C66" t="s">
-        <v>241</v>
+        <v>252</v>
       </c>
     </row>
     <row r="67" spans="1:3">
@@ -1847,10 +1856,10 @@
         <v>68</v>
       </c>
       <c r="B67" t="s">
-        <v>187</v>
+        <v>188</v>
       </c>
       <c r="C67" t="s">
-        <v>241</v>
+        <v>257</v>
       </c>
     </row>
     <row r="68" spans="1:3">
@@ -1858,10 +1867,10 @@
         <v>69</v>
       </c>
       <c r="B68" t="s">
-        <v>188</v>
+        <v>189</v>
       </c>
       <c r="C68" t="s">
-        <v>249</v>
+        <v>244</v>
       </c>
     </row>
     <row r="69" spans="1:3">
@@ -1869,10 +1878,10 @@
         <v>70</v>
       </c>
       <c r="B69" t="s">
-        <v>189</v>
+        <v>190</v>
       </c>
       <c r="C69" t="s">
-        <v>249</v>
+        <v>244</v>
       </c>
     </row>
     <row r="70" spans="1:3">
@@ -1880,10 +1889,10 @@
         <v>71</v>
       </c>
       <c r="B70" t="s">
-        <v>190</v>
+        <v>191</v>
       </c>
       <c r="C70" t="s">
-        <v>244</v>
+        <v>252</v>
       </c>
     </row>
     <row r="71" spans="1:3">
@@ -1891,10 +1900,10 @@
         <v>72</v>
       </c>
       <c r="B71" t="s">
-        <v>191</v>
+        <v>192</v>
       </c>
       <c r="C71" t="s">
-        <v>249</v>
+        <v>252</v>
       </c>
     </row>
     <row r="72" spans="1:3">
@@ -1902,10 +1911,10 @@
         <v>73</v>
       </c>
       <c r="B72" t="s">
-        <v>192</v>
+        <v>193</v>
       </c>
       <c r="C72" t="s">
-        <v>241</v>
+        <v>247</v>
       </c>
     </row>
     <row r="73" spans="1:3">
@@ -1913,10 +1922,10 @@
         <v>74</v>
       </c>
       <c r="B73" t="s">
-        <v>193</v>
+        <v>194</v>
       </c>
       <c r="C73" t="s">
-        <v>246</v>
+        <v>252</v>
       </c>
     </row>
     <row r="74" spans="1:3">
@@ -1924,10 +1933,10 @@
         <v>75</v>
       </c>
       <c r="B74" t="s">
-        <v>194</v>
+        <v>195</v>
       </c>
       <c r="C74" t="s">
-        <v>241</v>
+        <v>244</v>
       </c>
     </row>
     <row r="75" spans="1:3">
@@ -1935,10 +1944,10 @@
         <v>76</v>
       </c>
       <c r="B75" t="s">
-        <v>195</v>
+        <v>196</v>
       </c>
       <c r="C75" t="s">
-        <v>241</v>
+        <v>249</v>
       </c>
     </row>
     <row r="76" spans="1:3">
@@ -1946,10 +1955,10 @@
         <v>77</v>
       </c>
       <c r="B76" t="s">
-        <v>196</v>
+        <v>197</v>
       </c>
       <c r="C76" t="s">
-        <v>247</v>
+        <v>244</v>
       </c>
     </row>
     <row r="77" spans="1:3">
@@ -1957,10 +1966,10 @@
         <v>78</v>
       </c>
       <c r="B77" t="s">
-        <v>197</v>
+        <v>198</v>
       </c>
       <c r="C77" t="s">
-        <v>246</v>
+        <v>244</v>
       </c>
     </row>
     <row r="78" spans="1:3">
@@ -1968,10 +1977,10 @@
         <v>79</v>
       </c>
       <c r="B78" t="s">
-        <v>198</v>
+        <v>199</v>
       </c>
       <c r="C78" t="s">
-        <v>243</v>
+        <v>250</v>
       </c>
     </row>
     <row r="79" spans="1:3">
@@ -1979,10 +1988,10 @@
         <v>80</v>
       </c>
       <c r="B79" t="s">
-        <v>199</v>
+        <v>200</v>
       </c>
       <c r="C79" t="s">
-        <v>241</v>
+        <v>249</v>
       </c>
     </row>
     <row r="80" spans="1:3">
@@ -1990,10 +1999,10 @@
         <v>81</v>
       </c>
       <c r="B80" t="s">
-        <v>200</v>
+        <v>201</v>
       </c>
       <c r="C80" t="s">
-        <v>249</v>
+        <v>246</v>
       </c>
     </row>
     <row r="81" spans="1:3">
@@ -2001,10 +2010,10 @@
         <v>82</v>
       </c>
       <c r="B81" t="s">
-        <v>201</v>
+        <v>202</v>
       </c>
       <c r="C81" t="s">
-        <v>249</v>
+        <v>244</v>
       </c>
     </row>
     <row r="82" spans="1:3">
@@ -2012,10 +2021,10 @@
         <v>83</v>
       </c>
       <c r="B82" t="s">
-        <v>202</v>
+        <v>203</v>
       </c>
       <c r="C82" t="s">
-        <v>255</v>
+        <v>252</v>
       </c>
     </row>
     <row r="83" spans="1:3">
@@ -2023,10 +2032,10 @@
         <v>84</v>
       </c>
       <c r="B83" t="s">
-        <v>203</v>
+        <v>204</v>
       </c>
       <c r="C83" t="s">
-        <v>249</v>
+        <v>252</v>
       </c>
     </row>
     <row r="84" spans="1:3">
@@ -2034,10 +2043,10 @@
         <v>85</v>
       </c>
       <c r="B84" t="s">
-        <v>204</v>
+        <v>205</v>
       </c>
       <c r="C84" t="s">
-        <v>241</v>
+        <v>258</v>
       </c>
     </row>
     <row r="85" spans="1:3">
@@ -2045,10 +2054,10 @@
         <v>86</v>
       </c>
       <c r="B85" t="s">
-        <v>205</v>
+        <v>206</v>
       </c>
       <c r="C85" t="s">
-        <v>241</v>
+        <v>252</v>
       </c>
     </row>
     <row r="86" spans="1:3">
@@ -2056,10 +2065,10 @@
         <v>87</v>
       </c>
       <c r="B86" t="s">
-        <v>206</v>
+        <v>207</v>
       </c>
       <c r="C86" t="s">
-        <v>246</v>
+        <v>244</v>
       </c>
     </row>
     <row r="87" spans="1:3">
@@ -2067,10 +2076,10 @@
         <v>88</v>
       </c>
       <c r="B87" t="s">
-        <v>207</v>
+        <v>208</v>
       </c>
       <c r="C87" t="s">
-        <v>251</v>
+        <v>244</v>
       </c>
     </row>
     <row r="88" spans="1:3">
@@ -2078,7 +2087,7 @@
         <v>89</v>
       </c>
       <c r="B88" t="s">
-        <v>208</v>
+        <v>209</v>
       </c>
       <c r="C88" t="s">
         <v>249</v>
@@ -2089,10 +2098,10 @@
         <v>90</v>
       </c>
       <c r="B89" t="s">
-        <v>209</v>
+        <v>210</v>
       </c>
       <c r="C89" t="s">
-        <v>251</v>
+        <v>254</v>
       </c>
     </row>
     <row r="90" spans="1:3">
@@ -2100,10 +2109,10 @@
         <v>91</v>
       </c>
       <c r="B90" t="s">
-        <v>210</v>
+        <v>211</v>
       </c>
       <c r="C90" t="s">
-        <v>241</v>
+        <v>252</v>
       </c>
     </row>
     <row r="91" spans="1:3">
@@ -2111,10 +2120,10 @@
         <v>92</v>
       </c>
       <c r="B91" t="s">
-        <v>211</v>
+        <v>212</v>
       </c>
       <c r="C91" t="s">
-        <v>251</v>
+        <v>254</v>
       </c>
     </row>
     <row r="92" spans="1:3">
@@ -2122,10 +2131,10 @@
         <v>93</v>
       </c>
       <c r="B92" t="s">
-        <v>212</v>
+        <v>213</v>
       </c>
       <c r="C92" t="s">
-        <v>251</v>
+        <v>244</v>
       </c>
     </row>
     <row r="93" spans="1:3">
@@ -2133,10 +2142,10 @@
         <v>94</v>
       </c>
       <c r="B93" t="s">
-        <v>213</v>
+        <v>214</v>
       </c>
       <c r="C93" t="s">
-        <v>250</v>
+        <v>254</v>
       </c>
     </row>
     <row r="94" spans="1:3">
@@ -2144,10 +2153,10 @@
         <v>95</v>
       </c>
       <c r="B94" t="s">
-        <v>214</v>
+        <v>215</v>
       </c>
       <c r="C94" t="s">
-        <v>249</v>
+        <v>254</v>
       </c>
     </row>
     <row r="95" spans="1:3">
@@ -2155,10 +2164,10 @@
         <v>96</v>
       </c>
       <c r="B95" t="s">
-        <v>215</v>
+        <v>216</v>
       </c>
       <c r="C95" t="s">
-        <v>245</v>
+        <v>253</v>
       </c>
     </row>
     <row r="96" spans="1:3">
@@ -2166,10 +2175,10 @@
         <v>97</v>
       </c>
       <c r="B96" t="s">
-        <v>216</v>
+        <v>217</v>
       </c>
       <c r="C96" t="s">
-        <v>254</v>
+        <v>252</v>
       </c>
     </row>
     <row r="97" spans="1:3">
@@ -2177,10 +2186,10 @@
         <v>98</v>
       </c>
       <c r="B97" t="s">
-        <v>217</v>
+        <v>218</v>
       </c>
       <c r="C97" t="s">
-        <v>241</v>
+        <v>248</v>
       </c>
     </row>
     <row r="98" spans="1:3">
@@ -2188,10 +2197,10 @@
         <v>99</v>
       </c>
       <c r="B98" t="s">
-        <v>218</v>
+        <v>219</v>
       </c>
       <c r="C98" t="s">
-        <v>242</v>
+        <v>257</v>
       </c>
     </row>
     <row r="99" spans="1:3">
@@ -2199,10 +2208,10 @@
         <v>100</v>
       </c>
       <c r="B99" t="s">
-        <v>219</v>
+        <v>220</v>
       </c>
       <c r="C99" t="s">
-        <v>250</v>
+        <v>244</v>
       </c>
     </row>
     <row r="100" spans="1:3">
@@ -2210,10 +2219,10 @@
         <v>101</v>
       </c>
       <c r="B100" t="s">
-        <v>220</v>
+        <v>221</v>
       </c>
       <c r="C100" t="s">
-        <v>246</v>
+        <v>245</v>
       </c>
     </row>
     <row r="101" spans="1:3">
@@ -2221,10 +2230,10 @@
         <v>102</v>
       </c>
       <c r="B101" t="s">
-        <v>221</v>
+        <v>222</v>
       </c>
       <c r="C101" t="s">
-        <v>241</v>
+        <v>253</v>
       </c>
     </row>
     <row r="102" spans="1:3">
@@ -2232,10 +2241,10 @@
         <v>103</v>
       </c>
       <c r="B102" t="s">
-        <v>222</v>
+        <v>223</v>
       </c>
       <c r="C102" t="s">
-        <v>246</v>
+        <v>249</v>
       </c>
     </row>
     <row r="103" spans="1:3">
@@ -2243,7 +2252,7 @@
         <v>104</v>
       </c>
       <c r="B103" t="s">
-        <v>223</v>
+        <v>224</v>
       </c>
       <c r="C103" t="s">
         <v>244</v>
@@ -2254,10 +2263,10 @@
         <v>105</v>
       </c>
       <c r="B104" t="s">
-        <v>224</v>
+        <v>225</v>
       </c>
       <c r="C104" t="s">
-        <v>253</v>
+        <v>249</v>
       </c>
     </row>
     <row r="105" spans="1:3">
@@ -2265,10 +2274,10 @@
         <v>106</v>
       </c>
       <c r="B105" t="s">
-        <v>225</v>
+        <v>226</v>
       </c>
       <c r="C105" t="s">
-        <v>244</v>
+        <v>247</v>
       </c>
     </row>
     <row r="106" spans="1:3">
@@ -2276,10 +2285,10 @@
         <v>107</v>
       </c>
       <c r="B106" t="s">
-        <v>226</v>
+        <v>227</v>
       </c>
       <c r="C106" t="s">
-        <v>244</v>
+        <v>256</v>
       </c>
     </row>
     <row r="107" spans="1:3">
@@ -2287,10 +2296,10 @@
         <v>108</v>
       </c>
       <c r="B107" t="s">
-        <v>227</v>
+        <v>228</v>
       </c>
       <c r="C107" t="s">
-        <v>242</v>
+        <v>247</v>
       </c>
     </row>
     <row r="108" spans="1:3">
@@ -2298,10 +2307,10 @@
         <v>109</v>
       </c>
       <c r="B108" t="s">
-        <v>228</v>
+        <v>229</v>
       </c>
       <c r="C108" t="s">
-        <v>243</v>
+        <v>247</v>
       </c>
     </row>
     <row r="109" spans="1:3">
@@ -2309,10 +2318,10 @@
         <v>110</v>
       </c>
       <c r="B109" t="s">
-        <v>229</v>
+        <v>230</v>
       </c>
       <c r="C109" t="s">
-        <v>252</v>
+        <v>245</v>
       </c>
     </row>
     <row r="110" spans="1:3">
@@ -2320,10 +2329,10 @@
         <v>111</v>
       </c>
       <c r="B110" t="s">
-        <v>230</v>
+        <v>231</v>
       </c>
       <c r="C110" t="s">
-        <v>241</v>
+        <v>246</v>
       </c>
     </row>
     <row r="111" spans="1:3">
@@ -2331,10 +2340,10 @@
         <v>112</v>
       </c>
       <c r="B111" t="s">
-        <v>231</v>
+        <v>232</v>
       </c>
       <c r="C111" t="s">
-        <v>254</v>
+        <v>255</v>
       </c>
     </row>
     <row r="112" spans="1:3">
@@ -2342,10 +2351,10 @@
         <v>113</v>
       </c>
       <c r="B112" t="s">
-        <v>232</v>
+        <v>233</v>
       </c>
       <c r="C112" t="s">
-        <v>251</v>
+        <v>244</v>
       </c>
     </row>
     <row r="113" spans="1:3">
@@ -2353,10 +2362,10 @@
         <v>114</v>
       </c>
       <c r="B113" t="s">
-        <v>233</v>
+        <v>234</v>
       </c>
       <c r="C113" t="s">
-        <v>245</v>
+        <v>257</v>
       </c>
     </row>
     <row r="114" spans="1:3">
@@ -2364,10 +2373,10 @@
         <v>115</v>
       </c>
       <c r="B114" t="s">
-        <v>234</v>
+        <v>235</v>
       </c>
       <c r="C114" t="s">
-        <v>249</v>
+        <v>254</v>
       </c>
     </row>
     <row r="115" spans="1:3">
@@ -2375,10 +2384,10 @@
         <v>116</v>
       </c>
       <c r="B115" t="s">
-        <v>235</v>
+        <v>236</v>
       </c>
       <c r="C115" t="s">
-        <v>243</v>
+        <v>248</v>
       </c>
     </row>
     <row r="116" spans="1:3">
@@ -2386,10 +2395,10 @@
         <v>117</v>
       </c>
       <c r="B116" t="s">
-        <v>236</v>
+        <v>237</v>
       </c>
       <c r="C116" t="s">
-        <v>250</v>
+        <v>252</v>
       </c>
     </row>
     <row r="117" spans="1:3">
@@ -2397,10 +2406,10 @@
         <v>118</v>
       </c>
       <c r="B117" t="s">
-        <v>237</v>
+        <v>238</v>
       </c>
       <c r="C117" t="s">
-        <v>242</v>
+        <v>246</v>
       </c>
     </row>
     <row r="118" spans="1:3">
@@ -2408,10 +2417,10 @@
         <v>119</v>
       </c>
       <c r="B118" t="s">
-        <v>238</v>
+        <v>239</v>
       </c>
       <c r="C118" t="s">
-        <v>245</v>
+        <v>253</v>
       </c>
     </row>
     <row r="119" spans="1:3">
@@ -2419,10 +2428,10 @@
         <v>120</v>
       </c>
       <c r="B119" t="s">
-        <v>239</v>
+        <v>240</v>
       </c>
       <c r="C119" t="s">
-        <v>249</v>
+        <v>245</v>
       </c>
     </row>
     <row r="120" spans="1:3">
@@ -2430,10 +2439,32 @@
         <v>121</v>
       </c>
       <c r="B120" t="s">
-        <v>240</v>
+        <v>241</v>
       </c>
       <c r="C120" t="s">
-        <v>241</v>
+        <v>248</v>
+      </c>
+    </row>
+    <row r="121" spans="1:3">
+      <c r="A121" t="s">
+        <v>122</v>
+      </c>
+      <c r="B121" t="s">
+        <v>242</v>
+      </c>
+      <c r="C121" t="s">
+        <v>252</v>
+      </c>
+    </row>
+    <row r="122" spans="1:3">
+      <c r="A122" t="s">
+        <v>123</v>
+      </c>
+      <c r="B122" t="s">
+        <v>243</v>
+      </c>
+      <c r="C122" t="s">
+        <v>244</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Update student payments and add Ogunsanya records
Adjust payment totals and balances for multiple students in students_1st_term.json (e.g., ABIODUN DANIEL OBANIJESU, AKINDURO GABRIELLA, SANUSI JOSIAH). Add two new student entries OGUOLU1124 and OGUOPE1125 with full fee breakdowns. Add corresponding codes for these students to code_registry.json. Updated related binary spreadsheets (2026 - 2027 FEE.xlsx, parent_codes.xlsx) to reflect these changes.
</commit_message>
<xml_diff>
--- a/parent_codes.xlsx
+++ b/parent_codes.xlsx
@@ -14,7 +14,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="366" uniqueCount="259">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="371" uniqueCount="263">
   <si>
     <t>Code</t>
   </si>
@@ -271,6 +271,12 @@
     <t>OBETAI1079</t>
   </si>
   <si>
+    <t>OGUOLU1124</t>
+  </si>
+  <si>
+    <t>OGUOPE1125</t>
+  </si>
+  <si>
     <t>OKEJUM1081</t>
   </si>
   <si>
@@ -629,6 +635,12 @@
   </si>
   <si>
     <t>OBEY TAIWO EYITAYO</t>
+  </si>
+  <si>
+    <t>OGUNSANYA OLUWAFERANMI BLESSED</t>
+  </si>
+  <si>
+    <t>OGUNSANYA OPETOSIMI GRACE</t>
   </si>
   <si>
     <t>OKERINDE JUMAIN BOLUWATIFE</t>
@@ -1122,7 +1134,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C122"/>
+  <dimension ref="A1:C124"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:3">
@@ -1141,10 +1153,10 @@
         <v>3</v>
       </c>
       <c r="B2" t="s">
-        <v>124</v>
+        <v>126</v>
       </c>
       <c r="C2" t="s">
-        <v>244</v>
+        <v>248</v>
       </c>
     </row>
     <row r="3" spans="1:3">
@@ -1152,10 +1164,10 @@
         <v>4</v>
       </c>
       <c r="B3" t="s">
-        <v>125</v>
+        <v>127</v>
       </c>
       <c r="C3" t="s">
-        <v>245</v>
+        <v>249</v>
       </c>
     </row>
     <row r="4" spans="1:3">
@@ -1163,10 +1175,10 @@
         <v>5</v>
       </c>
       <c r="B4" t="s">
-        <v>126</v>
+        <v>128</v>
       </c>
       <c r="C4" t="s">
-        <v>246</v>
+        <v>250</v>
       </c>
     </row>
     <row r="5" spans="1:3">
@@ -1174,10 +1186,10 @@
         <v>6</v>
       </c>
       <c r="B5" t="s">
-        <v>127</v>
+        <v>129</v>
       </c>
       <c r="C5" t="s">
-        <v>247</v>
+        <v>251</v>
       </c>
     </row>
     <row r="6" spans="1:3">
@@ -1185,10 +1197,10 @@
         <v>7</v>
       </c>
       <c r="B6" t="s">
-        <v>128</v>
+        <v>130</v>
       </c>
       <c r="C6" t="s">
-        <v>244</v>
+        <v>248</v>
       </c>
     </row>
     <row r="7" spans="1:3">
@@ -1196,10 +1208,10 @@
         <v>8</v>
       </c>
       <c r="B7" t="s">
-        <v>129</v>
+        <v>131</v>
       </c>
       <c r="C7" t="s">
-        <v>248</v>
+        <v>252</v>
       </c>
     </row>
     <row r="8" spans="1:3">
@@ -1207,10 +1219,10 @@
         <v>9</v>
       </c>
       <c r="B8" t="s">
-        <v>130</v>
+        <v>132</v>
       </c>
       <c r="C8" t="s">
-        <v>249</v>
+        <v>253</v>
       </c>
     </row>
     <row r="9" spans="1:3">
@@ -1218,10 +1230,10 @@
         <v>10</v>
       </c>
       <c r="B9" t="s">
-        <v>131</v>
+        <v>133</v>
       </c>
       <c r="C9" t="s">
-        <v>248</v>
+        <v>252</v>
       </c>
     </row>
     <row r="10" spans="1:3">
@@ -1229,10 +1241,10 @@
         <v>11</v>
       </c>
       <c r="B10" t="s">
-        <v>132</v>
+        <v>134</v>
       </c>
       <c r="C10" t="s">
-        <v>248</v>
+        <v>252</v>
       </c>
     </row>
     <row r="11" spans="1:3">
@@ -1240,10 +1252,10 @@
         <v>12</v>
       </c>
       <c r="B11" t="s">
-        <v>133</v>
+        <v>135</v>
       </c>
       <c r="C11" t="s">
-        <v>248</v>
+        <v>252</v>
       </c>
     </row>
     <row r="12" spans="1:3">
@@ -1251,10 +1263,10 @@
         <v>13</v>
       </c>
       <c r="B12" t="s">
-        <v>134</v>
+        <v>136</v>
       </c>
       <c r="C12" t="s">
-        <v>247</v>
+        <v>251</v>
       </c>
     </row>
     <row r="13" spans="1:3">
@@ -1262,10 +1274,10 @@
         <v>14</v>
       </c>
       <c r="B13" t="s">
-        <v>135</v>
+        <v>137</v>
       </c>
       <c r="C13" t="s">
-        <v>249</v>
+        <v>253</v>
       </c>
     </row>
     <row r="14" spans="1:3">
@@ -1273,10 +1285,10 @@
         <v>15</v>
       </c>
       <c r="B14" t="s">
-        <v>136</v>
+        <v>138</v>
       </c>
       <c r="C14" t="s">
-        <v>246</v>
+        <v>250</v>
       </c>
     </row>
     <row r="15" spans="1:3">
@@ -1284,10 +1296,10 @@
         <v>16</v>
       </c>
       <c r="B15" t="s">
-        <v>137</v>
+        <v>139</v>
       </c>
       <c r="C15" t="s">
-        <v>245</v>
+        <v>249</v>
       </c>
     </row>
     <row r="16" spans="1:3">
@@ -1295,10 +1307,10 @@
         <v>17</v>
       </c>
       <c r="B16" t="s">
-        <v>138</v>
+        <v>140</v>
       </c>
       <c r="C16" t="s">
-        <v>249</v>
+        <v>253</v>
       </c>
     </row>
     <row r="17" spans="1:3">
@@ -1306,10 +1318,10 @@
         <v>18</v>
       </c>
       <c r="B17" t="s">
-        <v>139</v>
+        <v>141</v>
       </c>
       <c r="C17" t="s">
-        <v>247</v>
+        <v>251</v>
       </c>
     </row>
     <row r="18" spans="1:3">
@@ -1317,10 +1329,10 @@
         <v>19</v>
       </c>
       <c r="B18" t="s">
-        <v>140</v>
+        <v>142</v>
       </c>
       <c r="C18" t="s">
-        <v>250</v>
+        <v>254</v>
       </c>
     </row>
     <row r="19" spans="1:3">
@@ -1328,10 +1340,10 @@
         <v>20</v>
       </c>
       <c r="B19" t="s">
-        <v>141</v>
+        <v>143</v>
       </c>
       <c r="C19" t="s">
-        <v>245</v>
+        <v>249</v>
       </c>
     </row>
     <row r="20" spans="1:3">
@@ -1339,10 +1351,10 @@
         <v>21</v>
       </c>
       <c r="B20" t="s">
-        <v>142</v>
+        <v>144</v>
       </c>
       <c r="C20" t="s">
-        <v>251</v>
+        <v>255</v>
       </c>
     </row>
     <row r="21" spans="1:3">
@@ -1350,10 +1362,10 @@
         <v>22</v>
       </c>
       <c r="B21" t="s">
-        <v>143</v>
+        <v>145</v>
       </c>
       <c r="C21" t="s">
-        <v>248</v>
+        <v>252</v>
       </c>
     </row>
     <row r="22" spans="1:3">
@@ -1361,10 +1373,10 @@
         <v>23</v>
       </c>
       <c r="B22" t="s">
-        <v>144</v>
+        <v>146</v>
       </c>
       <c r="C22" t="s">
-        <v>252</v>
+        <v>256</v>
       </c>
     </row>
     <row r="23" spans="1:3">
@@ -1372,10 +1384,10 @@
         <v>24</v>
       </c>
       <c r="B23" t="s">
-        <v>145</v>
+        <v>147</v>
       </c>
       <c r="C23" t="s">
-        <v>253</v>
+        <v>257</v>
       </c>
     </row>
     <row r="24" spans="1:3">
@@ -1383,10 +1395,10 @@
         <v>25</v>
       </c>
       <c r="B24" t="s">
-        <v>146</v>
+        <v>148</v>
       </c>
       <c r="C24" t="s">
-        <v>252</v>
+        <v>256</v>
       </c>
     </row>
     <row r="25" spans="1:3">
@@ -1394,10 +1406,10 @@
         <v>26</v>
       </c>
       <c r="B25" t="s">
-        <v>147</v>
+        <v>149</v>
       </c>
       <c r="C25" t="s">
-        <v>248</v>
+        <v>252</v>
       </c>
     </row>
     <row r="26" spans="1:3">
@@ -1405,10 +1417,10 @@
         <v>27</v>
       </c>
       <c r="B26" t="s">
-        <v>148</v>
+        <v>150</v>
       </c>
       <c r="C26" t="s">
-        <v>254</v>
+        <v>258</v>
       </c>
     </row>
     <row r="27" spans="1:3">
@@ -1416,10 +1428,10 @@
         <v>28</v>
       </c>
       <c r="B27" t="s">
-        <v>149</v>
+        <v>151</v>
       </c>
       <c r="C27" t="s">
-        <v>253</v>
+        <v>257</v>
       </c>
     </row>
     <row r="28" spans="1:3">
@@ -1427,10 +1439,10 @@
         <v>29</v>
       </c>
       <c r="B28" t="s">
-        <v>150</v>
+        <v>152</v>
       </c>
       <c r="C28" t="s">
-        <v>255</v>
+        <v>259</v>
       </c>
     </row>
     <row r="29" spans="1:3">
@@ -1438,10 +1450,10 @@
         <v>30</v>
       </c>
       <c r="B29" t="s">
-        <v>151</v>
+        <v>153</v>
       </c>
       <c r="C29" t="s">
-        <v>250</v>
+        <v>254</v>
       </c>
     </row>
     <row r="30" spans="1:3">
@@ -1449,10 +1461,10 @@
         <v>31</v>
       </c>
       <c r="B30" t="s">
-        <v>152</v>
+        <v>154</v>
       </c>
       <c r="C30" t="s">
-        <v>250</v>
+        <v>254</v>
       </c>
     </row>
     <row r="31" spans="1:3">
@@ -1460,10 +1472,10 @@
         <v>32</v>
       </c>
       <c r="B31" t="s">
-        <v>153</v>
+        <v>155</v>
       </c>
       <c r="C31" t="s">
-        <v>252</v>
+        <v>256</v>
       </c>
     </row>
     <row r="32" spans="1:3">
@@ -1471,10 +1483,10 @@
         <v>33</v>
       </c>
       <c r="B32" t="s">
-        <v>154</v>
+        <v>156</v>
       </c>
       <c r="C32" t="s">
-        <v>256</v>
+        <v>260</v>
       </c>
     </row>
     <row r="33" spans="1:3">
@@ -1482,10 +1494,10 @@
         <v>34</v>
       </c>
       <c r="B33" t="s">
-        <v>155</v>
+        <v>157</v>
       </c>
       <c r="C33" t="s">
-        <v>244</v>
+        <v>248</v>
       </c>
     </row>
     <row r="34" spans="1:3">
@@ -1493,10 +1505,10 @@
         <v>35</v>
       </c>
       <c r="B34" t="s">
-        <v>156</v>
+        <v>158</v>
       </c>
       <c r="C34" t="s">
-        <v>245</v>
+        <v>249</v>
       </c>
     </row>
     <row r="35" spans="1:3">
@@ -1504,10 +1516,10 @@
         <v>36</v>
       </c>
       <c r="B35" t="s">
-        <v>157</v>
+        <v>159</v>
       </c>
       <c r="C35" t="s">
-        <v>244</v>
+        <v>248</v>
       </c>
     </row>
     <row r="36" spans="1:3">
@@ -1515,10 +1527,10 @@
         <v>37</v>
       </c>
       <c r="B36" t="s">
-        <v>158</v>
+        <v>160</v>
       </c>
       <c r="C36" t="s">
-        <v>247</v>
+        <v>251</v>
       </c>
     </row>
     <row r="37" spans="1:3">
@@ -1526,10 +1538,10 @@
         <v>38</v>
       </c>
       <c r="B37" t="s">
-        <v>159</v>
+        <v>161</v>
       </c>
       <c r="C37" t="s">
-        <v>252</v>
+        <v>256</v>
       </c>
     </row>
     <row r="38" spans="1:3">
@@ -1537,10 +1549,10 @@
         <v>39</v>
       </c>
       <c r="B38" t="s">
-        <v>160</v>
+        <v>162</v>
       </c>
       <c r="C38" t="s">
-        <v>256</v>
+        <v>260</v>
       </c>
     </row>
     <row r="39" spans="1:3">
@@ -1548,10 +1560,10 @@
         <v>40</v>
       </c>
       <c r="B39" t="s">
-        <v>161</v>
+        <v>163</v>
       </c>
       <c r="C39" t="s">
-        <v>252</v>
+        <v>256</v>
       </c>
     </row>
     <row r="40" spans="1:3">
@@ -1559,10 +1571,10 @@
         <v>41</v>
       </c>
       <c r="B40" t="s">
-        <v>162</v>
+        <v>164</v>
       </c>
       <c r="C40" t="s">
-        <v>253</v>
+        <v>257</v>
       </c>
     </row>
     <row r="41" spans="1:3">
@@ -1570,10 +1582,10 @@
         <v>42</v>
       </c>
       <c r="B41" t="s">
-        <v>163</v>
+        <v>165</v>
       </c>
       <c r="C41" t="s">
-        <v>253</v>
+        <v>257</v>
       </c>
     </row>
     <row r="42" spans="1:3">
@@ -1581,10 +1593,10 @@
         <v>43</v>
       </c>
       <c r="B42" t="s">
-        <v>164</v>
+        <v>166</v>
       </c>
       <c r="C42" t="s">
-        <v>246</v>
+        <v>250</v>
       </c>
     </row>
     <row r="43" spans="1:3">
@@ -1592,10 +1604,10 @@
         <v>44</v>
       </c>
       <c r="B43" t="s">
-        <v>165</v>
+        <v>167</v>
       </c>
       <c r="C43" t="s">
-        <v>253</v>
+        <v>257</v>
       </c>
     </row>
     <row r="44" spans="1:3">
@@ -1603,10 +1615,10 @@
         <v>45</v>
       </c>
       <c r="B44" t="s">
-        <v>166</v>
+        <v>168</v>
       </c>
       <c r="C44" t="s">
-        <v>253</v>
+        <v>257</v>
       </c>
     </row>
     <row r="45" spans="1:3">
@@ -1614,10 +1626,10 @@
         <v>46</v>
       </c>
       <c r="B45" t="s">
-        <v>167</v>
+        <v>169</v>
       </c>
       <c r="C45" t="s">
-        <v>246</v>
+        <v>250</v>
       </c>
     </row>
     <row r="46" spans="1:3">
@@ -1625,10 +1637,10 @@
         <v>47</v>
       </c>
       <c r="B46" t="s">
-        <v>168</v>
+        <v>170</v>
       </c>
       <c r="C46" t="s">
-        <v>252</v>
+        <v>256</v>
       </c>
     </row>
     <row r="47" spans="1:3">
@@ -1636,10 +1648,10 @@
         <v>48</v>
       </c>
       <c r="B47" t="s">
-        <v>169</v>
+        <v>171</v>
       </c>
       <c r="C47" t="s">
-        <v>255</v>
+        <v>259</v>
       </c>
     </row>
     <row r="48" spans="1:3">
@@ -1647,10 +1659,10 @@
         <v>49</v>
       </c>
       <c r="B48" t="s">
-        <v>170</v>
+        <v>172</v>
       </c>
       <c r="C48" t="s">
-        <v>247</v>
+        <v>251</v>
       </c>
     </row>
     <row r="49" spans="1:3">
@@ -1658,10 +1670,10 @@
         <v>50</v>
       </c>
       <c r="B49" t="s">
-        <v>171</v>
+        <v>173</v>
       </c>
       <c r="C49" t="s">
-        <v>254</v>
+        <v>258</v>
       </c>
     </row>
     <row r="50" spans="1:3">
@@ -1669,10 +1681,10 @@
         <v>51</v>
       </c>
       <c r="B50" t="s">
-        <v>172</v>
+        <v>174</v>
       </c>
       <c r="C50" t="s">
-        <v>253</v>
+        <v>257</v>
       </c>
     </row>
     <row r="51" spans="1:3">
@@ -1680,10 +1692,10 @@
         <v>52</v>
       </c>
       <c r="B51" t="s">
-        <v>173</v>
+        <v>175</v>
       </c>
       <c r="C51" t="s">
-        <v>255</v>
+        <v>259</v>
       </c>
     </row>
     <row r="52" spans="1:3">
@@ -1691,10 +1703,10 @@
         <v>53</v>
       </c>
       <c r="B52" t="s">
-        <v>174</v>
+        <v>176</v>
       </c>
       <c r="C52" t="s">
-        <v>245</v>
+        <v>249</v>
       </c>
     </row>
     <row r="53" spans="1:3">
@@ -1702,10 +1714,10 @@
         <v>54</v>
       </c>
       <c r="B53" t="s">
-        <v>175</v>
+        <v>177</v>
       </c>
       <c r="C53" t="s">
-        <v>248</v>
+        <v>252</v>
       </c>
     </row>
     <row r="54" spans="1:3">
@@ -1713,10 +1725,10 @@
         <v>55</v>
       </c>
       <c r="B54" t="s">
-        <v>176</v>
+        <v>178</v>
       </c>
       <c r="C54" t="s">
-        <v>252</v>
+        <v>256</v>
       </c>
     </row>
     <row r="55" spans="1:3">
@@ -1724,10 +1736,10 @@
         <v>56</v>
       </c>
       <c r="B55" t="s">
-        <v>177</v>
+        <v>179</v>
       </c>
       <c r="C55" t="s">
-        <v>253</v>
+        <v>257</v>
       </c>
     </row>
     <row r="56" spans="1:3">
@@ -1735,10 +1747,10 @@
         <v>57</v>
       </c>
       <c r="B56" t="s">
-        <v>177</v>
+        <v>179</v>
       </c>
       <c r="C56" t="s">
-        <v>251</v>
+        <v>255</v>
       </c>
     </row>
     <row r="57" spans="1:3">
@@ -1746,10 +1758,10 @@
         <v>58</v>
       </c>
       <c r="B57" t="s">
-        <v>178</v>
+        <v>180</v>
       </c>
       <c r="C57" t="s">
-        <v>244</v>
+        <v>248</v>
       </c>
     </row>
     <row r="58" spans="1:3">
@@ -1757,10 +1769,10 @@
         <v>59</v>
       </c>
       <c r="B58" t="s">
-        <v>179</v>
+        <v>181</v>
       </c>
       <c r="C58" t="s">
-        <v>254</v>
+        <v>258</v>
       </c>
     </row>
     <row r="59" spans="1:3">
@@ -1768,10 +1780,10 @@
         <v>60</v>
       </c>
       <c r="B59" t="s">
-        <v>180</v>
+        <v>182</v>
       </c>
       <c r="C59" t="s">
-        <v>244</v>
+        <v>248</v>
       </c>
     </row>
     <row r="60" spans="1:3">
@@ -1779,10 +1791,10 @@
         <v>61</v>
       </c>
       <c r="B60" t="s">
-        <v>181</v>
+        <v>183</v>
       </c>
       <c r="C60" t="s">
-        <v>244</v>
+        <v>248</v>
       </c>
     </row>
     <row r="61" spans="1:3">
@@ -1790,10 +1802,10 @@
         <v>62</v>
       </c>
       <c r="B61" t="s">
-        <v>182</v>
+        <v>184</v>
       </c>
       <c r="C61" t="s">
-        <v>254</v>
+        <v>258</v>
       </c>
     </row>
     <row r="62" spans="1:3">
@@ -1801,10 +1813,10 @@
         <v>63</v>
       </c>
       <c r="B62" t="s">
-        <v>183</v>
+        <v>185</v>
       </c>
       <c r="C62" t="s">
-        <v>249</v>
+        <v>253</v>
       </c>
     </row>
     <row r="63" spans="1:3">
@@ -1812,10 +1824,10 @@
         <v>64</v>
       </c>
       <c r="B63" t="s">
-        <v>184</v>
+        <v>186</v>
       </c>
       <c r="C63" t="s">
-        <v>253</v>
+        <v>257</v>
       </c>
     </row>
     <row r="64" spans="1:3">
@@ -1823,10 +1835,10 @@
         <v>65</v>
       </c>
       <c r="B64" t="s">
-        <v>185</v>
+        <v>187</v>
       </c>
       <c r="C64" t="s">
-        <v>257</v>
+        <v>261</v>
       </c>
     </row>
     <row r="65" spans="1:3">
@@ -1834,10 +1846,10 @@
         <v>66</v>
       </c>
       <c r="B65" t="s">
-        <v>186</v>
+        <v>188</v>
       </c>
       <c r="C65" t="s">
-        <v>250</v>
+        <v>254</v>
       </c>
     </row>
     <row r="66" spans="1:3">
@@ -1845,10 +1857,10 @@
         <v>67</v>
       </c>
       <c r="B66" t="s">
-        <v>187</v>
+        <v>189</v>
       </c>
       <c r="C66" t="s">
-        <v>252</v>
+        <v>256</v>
       </c>
     </row>
     <row r="67" spans="1:3">
@@ -1856,10 +1868,10 @@
         <v>68</v>
       </c>
       <c r="B67" t="s">
-        <v>188</v>
+        <v>190</v>
       </c>
       <c r="C67" t="s">
-        <v>257</v>
+        <v>261</v>
       </c>
     </row>
     <row r="68" spans="1:3">
@@ -1867,10 +1879,10 @@
         <v>69</v>
       </c>
       <c r="B68" t="s">
-        <v>189</v>
+        <v>191</v>
       </c>
       <c r="C68" t="s">
-        <v>244</v>
+        <v>248</v>
       </c>
     </row>
     <row r="69" spans="1:3">
@@ -1878,10 +1890,10 @@
         <v>70</v>
       </c>
       <c r="B69" t="s">
-        <v>190</v>
+        <v>192</v>
       </c>
       <c r="C69" t="s">
-        <v>244</v>
+        <v>248</v>
       </c>
     </row>
     <row r="70" spans="1:3">
@@ -1889,10 +1901,10 @@
         <v>71</v>
       </c>
       <c r="B70" t="s">
-        <v>191</v>
+        <v>193</v>
       </c>
       <c r="C70" t="s">
-        <v>252</v>
+        <v>256</v>
       </c>
     </row>
     <row r="71" spans="1:3">
@@ -1900,10 +1912,10 @@
         <v>72</v>
       </c>
       <c r="B71" t="s">
-        <v>192</v>
+        <v>194</v>
       </c>
       <c r="C71" t="s">
-        <v>252</v>
+        <v>256</v>
       </c>
     </row>
     <row r="72" spans="1:3">
@@ -1911,10 +1923,10 @@
         <v>73</v>
       </c>
       <c r="B72" t="s">
-        <v>193</v>
+        <v>195</v>
       </c>
       <c r="C72" t="s">
-        <v>247</v>
+        <v>251</v>
       </c>
     </row>
     <row r="73" spans="1:3">
@@ -1922,10 +1934,10 @@
         <v>74</v>
       </c>
       <c r="B73" t="s">
-        <v>194</v>
+        <v>196</v>
       </c>
       <c r="C73" t="s">
-        <v>252</v>
+        <v>256</v>
       </c>
     </row>
     <row r="74" spans="1:3">
@@ -1933,10 +1945,10 @@
         <v>75</v>
       </c>
       <c r="B74" t="s">
-        <v>195</v>
+        <v>197</v>
       </c>
       <c r="C74" t="s">
-        <v>244</v>
+        <v>248</v>
       </c>
     </row>
     <row r="75" spans="1:3">
@@ -1944,10 +1956,10 @@
         <v>76</v>
       </c>
       <c r="B75" t="s">
-        <v>196</v>
+        <v>198</v>
       </c>
       <c r="C75" t="s">
-        <v>249</v>
+        <v>253</v>
       </c>
     </row>
     <row r="76" spans="1:3">
@@ -1955,10 +1967,10 @@
         <v>77</v>
       </c>
       <c r="B76" t="s">
-        <v>197</v>
+        <v>199</v>
       </c>
       <c r="C76" t="s">
-        <v>244</v>
+        <v>248</v>
       </c>
     </row>
     <row r="77" spans="1:3">
@@ -1966,10 +1978,10 @@
         <v>78</v>
       </c>
       <c r="B77" t="s">
-        <v>198</v>
+        <v>200</v>
       </c>
       <c r="C77" t="s">
-        <v>244</v>
+        <v>248</v>
       </c>
     </row>
     <row r="78" spans="1:3">
@@ -1977,10 +1989,10 @@
         <v>79</v>
       </c>
       <c r="B78" t="s">
-        <v>199</v>
+        <v>201</v>
       </c>
       <c r="C78" t="s">
-        <v>250</v>
+        <v>254</v>
       </c>
     </row>
     <row r="79" spans="1:3">
@@ -1988,10 +2000,10 @@
         <v>80</v>
       </c>
       <c r="B79" t="s">
-        <v>200</v>
+        <v>202</v>
       </c>
       <c r="C79" t="s">
-        <v>249</v>
+        <v>253</v>
       </c>
     </row>
     <row r="80" spans="1:3">
@@ -1999,10 +2011,10 @@
         <v>81</v>
       </c>
       <c r="B80" t="s">
-        <v>201</v>
+        <v>203</v>
       </c>
       <c r="C80" t="s">
-        <v>246</v>
+        <v>250</v>
       </c>
     </row>
     <row r="81" spans="1:3">
@@ -2010,10 +2022,10 @@
         <v>82</v>
       </c>
       <c r="B81" t="s">
-        <v>202</v>
+        <v>204</v>
       </c>
       <c r="C81" t="s">
-        <v>244</v>
+        <v>248</v>
       </c>
     </row>
     <row r="82" spans="1:3">
@@ -2021,10 +2033,10 @@
         <v>83</v>
       </c>
       <c r="B82" t="s">
-        <v>203</v>
+        <v>205</v>
       </c>
       <c r="C82" t="s">
-        <v>252</v>
+        <v>256</v>
       </c>
     </row>
     <row r="83" spans="1:3">
@@ -2032,10 +2044,10 @@
         <v>84</v>
       </c>
       <c r="B83" t="s">
-        <v>204</v>
+        <v>206</v>
       </c>
       <c r="C83" t="s">
-        <v>252</v>
+        <v>256</v>
       </c>
     </row>
     <row r="84" spans="1:3">
@@ -2043,10 +2055,10 @@
         <v>85</v>
       </c>
       <c r="B84" t="s">
-        <v>205</v>
+        <v>207</v>
       </c>
       <c r="C84" t="s">
-        <v>258</v>
+        <v>252</v>
       </c>
     </row>
     <row r="85" spans="1:3">
@@ -2054,10 +2066,7 @@
         <v>86</v>
       </c>
       <c r="B85" t="s">
-        <v>206</v>
-      </c>
-      <c r="C85" t="s">
-        <v>252</v>
+        <v>208</v>
       </c>
     </row>
     <row r="86" spans="1:3">
@@ -2065,10 +2074,10 @@
         <v>87</v>
       </c>
       <c r="B86" t="s">
-        <v>207</v>
+        <v>209</v>
       </c>
       <c r="C86" t="s">
-        <v>244</v>
+        <v>262</v>
       </c>
     </row>
     <row r="87" spans="1:3">
@@ -2076,10 +2085,10 @@
         <v>88</v>
       </c>
       <c r="B87" t="s">
-        <v>208</v>
+        <v>210</v>
       </c>
       <c r="C87" t="s">
-        <v>244</v>
+        <v>256</v>
       </c>
     </row>
     <row r="88" spans="1:3">
@@ -2087,10 +2096,10 @@
         <v>89</v>
       </c>
       <c r="B88" t="s">
-        <v>209</v>
+        <v>211</v>
       </c>
       <c r="C88" t="s">
-        <v>249</v>
+        <v>248</v>
       </c>
     </row>
     <row r="89" spans="1:3">
@@ -2098,10 +2107,10 @@
         <v>90</v>
       </c>
       <c r="B89" t="s">
-        <v>210</v>
+        <v>212</v>
       </c>
       <c r="C89" t="s">
-        <v>254</v>
+        <v>248</v>
       </c>
     </row>
     <row r="90" spans="1:3">
@@ -2109,10 +2118,10 @@
         <v>91</v>
       </c>
       <c r="B90" t="s">
-        <v>211</v>
+        <v>213</v>
       </c>
       <c r="C90" t="s">
-        <v>252</v>
+        <v>253</v>
       </c>
     </row>
     <row r="91" spans="1:3">
@@ -2120,10 +2129,10 @@
         <v>92</v>
       </c>
       <c r="B91" t="s">
-        <v>212</v>
+        <v>214</v>
       </c>
       <c r="C91" t="s">
-        <v>254</v>
+        <v>258</v>
       </c>
     </row>
     <row r="92" spans="1:3">
@@ -2131,10 +2140,10 @@
         <v>93</v>
       </c>
       <c r="B92" t="s">
-        <v>213</v>
+        <v>215</v>
       </c>
       <c r="C92" t="s">
-        <v>244</v>
+        <v>256</v>
       </c>
     </row>
     <row r="93" spans="1:3">
@@ -2142,10 +2151,10 @@
         <v>94</v>
       </c>
       <c r="B93" t="s">
-        <v>214</v>
+        <v>216</v>
       </c>
       <c r="C93" t="s">
-        <v>254</v>
+        <v>258</v>
       </c>
     </row>
     <row r="94" spans="1:3">
@@ -2153,10 +2162,10 @@
         <v>95</v>
       </c>
       <c r="B94" t="s">
-        <v>215</v>
+        <v>217</v>
       </c>
       <c r="C94" t="s">
-        <v>254</v>
+        <v>248</v>
       </c>
     </row>
     <row r="95" spans="1:3">
@@ -2164,10 +2173,10 @@
         <v>96</v>
       </c>
       <c r="B95" t="s">
-        <v>216</v>
+        <v>218</v>
       </c>
       <c r="C95" t="s">
-        <v>253</v>
+        <v>258</v>
       </c>
     </row>
     <row r="96" spans="1:3">
@@ -2175,10 +2184,10 @@
         <v>97</v>
       </c>
       <c r="B96" t="s">
-        <v>217</v>
+        <v>219</v>
       </c>
       <c r="C96" t="s">
-        <v>252</v>
+        <v>258</v>
       </c>
     </row>
     <row r="97" spans="1:3">
@@ -2186,10 +2195,10 @@
         <v>98</v>
       </c>
       <c r="B97" t="s">
-        <v>218</v>
+        <v>220</v>
       </c>
       <c r="C97" t="s">
-        <v>248</v>
+        <v>257</v>
       </c>
     </row>
     <row r="98" spans="1:3">
@@ -2197,10 +2206,10 @@
         <v>99</v>
       </c>
       <c r="B98" t="s">
-        <v>219</v>
+        <v>221</v>
       </c>
       <c r="C98" t="s">
-        <v>257</v>
+        <v>256</v>
       </c>
     </row>
     <row r="99" spans="1:3">
@@ -2208,10 +2217,10 @@
         <v>100</v>
       </c>
       <c r="B99" t="s">
-        <v>220</v>
+        <v>222</v>
       </c>
       <c r="C99" t="s">
-        <v>244</v>
+        <v>252</v>
       </c>
     </row>
     <row r="100" spans="1:3">
@@ -2219,10 +2228,10 @@
         <v>101</v>
       </c>
       <c r="B100" t="s">
-        <v>221</v>
+        <v>223</v>
       </c>
       <c r="C100" t="s">
-        <v>245</v>
+        <v>261</v>
       </c>
     </row>
     <row r="101" spans="1:3">
@@ -2230,10 +2239,10 @@
         <v>102</v>
       </c>
       <c r="B101" t="s">
-        <v>222</v>
+        <v>224</v>
       </c>
       <c r="C101" t="s">
-        <v>253</v>
+        <v>248</v>
       </c>
     </row>
     <row r="102" spans="1:3">
@@ -2241,7 +2250,7 @@
         <v>103</v>
       </c>
       <c r="B102" t="s">
-        <v>223</v>
+        <v>225</v>
       </c>
       <c r="C102" t="s">
         <v>249</v>
@@ -2252,10 +2261,10 @@
         <v>104</v>
       </c>
       <c r="B103" t="s">
-        <v>224</v>
+        <v>226</v>
       </c>
       <c r="C103" t="s">
-        <v>244</v>
+        <v>257</v>
       </c>
     </row>
     <row r="104" spans="1:3">
@@ -2263,10 +2272,10 @@
         <v>105</v>
       </c>
       <c r="B104" t="s">
-        <v>225</v>
+        <v>227</v>
       </c>
       <c r="C104" t="s">
-        <v>249</v>
+        <v>253</v>
       </c>
     </row>
     <row r="105" spans="1:3">
@@ -2274,10 +2283,10 @@
         <v>106</v>
       </c>
       <c r="B105" t="s">
-        <v>226</v>
+        <v>228</v>
       </c>
       <c r="C105" t="s">
-        <v>247</v>
+        <v>248</v>
       </c>
     </row>
     <row r="106" spans="1:3">
@@ -2285,10 +2294,10 @@
         <v>107</v>
       </c>
       <c r="B106" t="s">
-        <v>227</v>
+        <v>229</v>
       </c>
       <c r="C106" t="s">
-        <v>256</v>
+        <v>253</v>
       </c>
     </row>
     <row r="107" spans="1:3">
@@ -2296,10 +2305,10 @@
         <v>108</v>
       </c>
       <c r="B107" t="s">
-        <v>228</v>
+        <v>230</v>
       </c>
       <c r="C107" t="s">
-        <v>247</v>
+        <v>251</v>
       </c>
     </row>
     <row r="108" spans="1:3">
@@ -2307,10 +2316,10 @@
         <v>109</v>
       </c>
       <c r="B108" t="s">
-        <v>229</v>
+        <v>231</v>
       </c>
       <c r="C108" t="s">
-        <v>247</v>
+        <v>260</v>
       </c>
     </row>
     <row r="109" spans="1:3">
@@ -2318,10 +2327,10 @@
         <v>110</v>
       </c>
       <c r="B109" t="s">
-        <v>230</v>
+        <v>232</v>
       </c>
       <c r="C109" t="s">
-        <v>245</v>
+        <v>251</v>
       </c>
     </row>
     <row r="110" spans="1:3">
@@ -2329,10 +2338,10 @@
         <v>111</v>
       </c>
       <c r="B110" t="s">
-        <v>231</v>
+        <v>233</v>
       </c>
       <c r="C110" t="s">
-        <v>246</v>
+        <v>251</v>
       </c>
     </row>
     <row r="111" spans="1:3">
@@ -2340,10 +2349,10 @@
         <v>112</v>
       </c>
       <c r="B111" t="s">
-        <v>232</v>
+        <v>234</v>
       </c>
       <c r="C111" t="s">
-        <v>255</v>
+        <v>249</v>
       </c>
     </row>
     <row r="112" spans="1:3">
@@ -2351,10 +2360,10 @@
         <v>113</v>
       </c>
       <c r="B112" t="s">
-        <v>233</v>
+        <v>235</v>
       </c>
       <c r="C112" t="s">
-        <v>244</v>
+        <v>250</v>
       </c>
     </row>
     <row r="113" spans="1:3">
@@ -2362,10 +2371,10 @@
         <v>114</v>
       </c>
       <c r="B113" t="s">
-        <v>234</v>
+        <v>236</v>
       </c>
       <c r="C113" t="s">
-        <v>257</v>
+        <v>259</v>
       </c>
     </row>
     <row r="114" spans="1:3">
@@ -2373,10 +2382,10 @@
         <v>115</v>
       </c>
       <c r="B114" t="s">
-        <v>235</v>
+        <v>237</v>
       </c>
       <c r="C114" t="s">
-        <v>254</v>
+        <v>248</v>
       </c>
     </row>
     <row r="115" spans="1:3">
@@ -2384,10 +2393,10 @@
         <v>116</v>
       </c>
       <c r="B115" t="s">
-        <v>236</v>
+        <v>238</v>
       </c>
       <c r="C115" t="s">
-        <v>248</v>
+        <v>261</v>
       </c>
     </row>
     <row r="116" spans="1:3">
@@ -2395,10 +2404,10 @@
         <v>117</v>
       </c>
       <c r="B116" t="s">
-        <v>237</v>
+        <v>239</v>
       </c>
       <c r="C116" t="s">
-        <v>252</v>
+        <v>258</v>
       </c>
     </row>
     <row r="117" spans="1:3">
@@ -2406,10 +2415,10 @@
         <v>118</v>
       </c>
       <c r="B117" t="s">
-        <v>238</v>
+        <v>240</v>
       </c>
       <c r="C117" t="s">
-        <v>246</v>
+        <v>252</v>
       </c>
     </row>
     <row r="118" spans="1:3">
@@ -2417,10 +2426,10 @@
         <v>119</v>
       </c>
       <c r="B118" t="s">
-        <v>239</v>
+        <v>241</v>
       </c>
       <c r="C118" t="s">
-        <v>253</v>
+        <v>256</v>
       </c>
     </row>
     <row r="119" spans="1:3">
@@ -2428,10 +2437,10 @@
         <v>120</v>
       </c>
       <c r="B119" t="s">
-        <v>240</v>
+        <v>242</v>
       </c>
       <c r="C119" t="s">
-        <v>245</v>
+        <v>250</v>
       </c>
     </row>
     <row r="120" spans="1:3">
@@ -2439,10 +2448,10 @@
         <v>121</v>
       </c>
       <c r="B120" t="s">
-        <v>241</v>
+        <v>243</v>
       </c>
       <c r="C120" t="s">
-        <v>248</v>
+        <v>257</v>
       </c>
     </row>
     <row r="121" spans="1:3">
@@ -2450,10 +2459,10 @@
         <v>122</v>
       </c>
       <c r="B121" t="s">
-        <v>242</v>
+        <v>244</v>
       </c>
       <c r="C121" t="s">
-        <v>252</v>
+        <v>249</v>
       </c>
     </row>
     <row r="122" spans="1:3">
@@ -2461,10 +2470,32 @@
         <v>123</v>
       </c>
       <c r="B122" t="s">
-        <v>243</v>
+        <v>245</v>
       </c>
       <c r="C122" t="s">
-        <v>244</v>
+        <v>252</v>
+      </c>
+    </row>
+    <row r="123" spans="1:3">
+      <c r="A123" t="s">
+        <v>124</v>
+      </c>
+      <c r="B123" t="s">
+        <v>246</v>
+      </c>
+      <c r="C123" t="s">
+        <v>256</v>
+      </c>
+    </row>
+    <row r="124" spans="1:3">
+      <c r="A124" t="s">
+        <v>125</v>
+      </c>
+      <c r="B124" t="s">
+        <v>247</v>
+      </c>
+      <c r="C124" t="s">
+        <v>248</v>
       </c>
     </row>
   </sheetData>

</xml_diff>